<commit_message>
founded base for teachers changes.  done create_class_teacher_subject_connetions, create_schedule_from_file in progress
</commit_message>
<xml_diff>
--- a/current_version_schedules/расписание в учительскую.xlsx
+++ b/current_version_schedules/расписание в учительскую.xlsx
@@ -2139,10 +2139,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2447,444 +2447,444 @@
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
     <col min="2" max="2" width="17.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="46" width="8.88671875" style="2" customWidth="1"/>
+    <col min="3" max="46" width="8.88671875" style="2" hidden="1" customWidth="1"/>
     <col min="47" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
-      <c r="AA1" s="3"/>
-      <c r="AB1" s="3"/>
-      <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AI1" s="3"/>
-      <c r="AJ1" s="3"/>
-      <c r="AK1" s="3"/>
-      <c r="AL1" s="3"/>
-      <c r="AM1" s="3"/>
-      <c r="AN1" s="3"/>
-      <c r="AO1" s="3"/>
-      <c r="AP1" s="3"/>
-      <c r="AQ1" s="3"/>
-      <c r="AR1" s="3"/>
-      <c r="AS1" s="3"/>
-      <c r="AT1" s="3"/>
-      <c r="AU1" s="3"/>
-      <c r="AV1" s="3"/>
-      <c r="AW1" s="3"/>
-      <c r="AX1" s="3"/>
-      <c r="AY1" s="3"/>
-      <c r="AZ1" s="3"/>
-      <c r="BA1" s="3"/>
-      <c r="BB1" s="3"/>
-      <c r="BC1" s="3"/>
-      <c r="BD1" s="3"/>
-      <c r="BE1" s="3"/>
-      <c r="BF1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
+      <c r="AP1" s="4"/>
+      <c r="AQ1" s="4"/>
+      <c r="AR1" s="4"/>
+      <c r="AS1" s="4"/>
+      <c r="AT1" s="4"/>
+      <c r="AU1" s="4"/>
+      <c r="AV1" s="4"/>
+      <c r="AW1" s="4"/>
+      <c r="AX1" s="4"/>
+      <c r="AY1" s="4"/>
+      <c r="AZ1" s="4"/>
+      <c r="BA1" s="4"/>
+      <c r="BB1" s="4"/>
+      <c r="BC1" s="4"/>
+      <c r="BD1" s="4"/>
+      <c r="BE1" s="4"/>
+      <c r="BF1" s="4"/>
     </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
-      <c r="Z2" s="3"/>
-      <c r="AA2" s="3"/>
-      <c r="AB2" s="3"/>
-      <c r="AC2" s="3"/>
-      <c r="AD2" s="3"/>
-      <c r="AE2" s="3"/>
-      <c r="AF2" s="3"/>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="3"/>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-      <c r="AK2" s="3"/>
-      <c r="AL2" s="3"/>
-      <c r="AM2" s="3"/>
-      <c r="AN2" s="3"/>
-      <c r="AO2" s="3"/>
-      <c r="AP2" s="3"/>
-      <c r="AQ2" s="3"/>
-      <c r="AR2" s="3"/>
-      <c r="AS2" s="3"/>
-      <c r="AT2" s="3"/>
-      <c r="AU2" s="3"/>
-      <c r="AV2" s="3"/>
-      <c r="AW2" s="3"/>
-      <c r="AX2" s="3"/>
-      <c r="AY2" s="3"/>
-      <c r="AZ2" s="3"/>
-      <c r="BA2" s="3"/>
-      <c r="BB2" s="3"/>
-      <c r="BC2" s="3"/>
-      <c r="BD2" s="3"/>
-      <c r="BE2" s="3"/>
-      <c r="BF2" s="3"/>
+    <row r="2" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
+      <c r="AG2" s="4"/>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="4"/>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
+      <c r="AL2" s="4"/>
+      <c r="AM2" s="4"/>
+      <c r="AN2" s="4"/>
+      <c r="AO2" s="4"/>
+      <c r="AP2" s="4"/>
+      <c r="AQ2" s="4"/>
+      <c r="AR2" s="4"/>
+      <c r="AS2" s="4"/>
+      <c r="AT2" s="4"/>
+      <c r="AU2" s="4"/>
+      <c r="AV2" s="4"/>
+      <c r="AW2" s="4"/>
+      <c r="AX2" s="4"/>
+      <c r="AY2" s="4"/>
+      <c r="AZ2" s="4"/>
+      <c r="BA2" s="4"/>
+      <c r="BB2" s="4"/>
+      <c r="BC2" s="4"/>
+      <c r="BD2" s="4"/>
+      <c r="BE2" s="4"/>
+      <c r="BF2" s="4"/>
     </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
-      <c r="AE3" s="3"/>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3"/>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
-      <c r="AK3" s="3"/>
-      <c r="AL3" s="3"/>
-      <c r="AM3" s="3"/>
-      <c r="AN3" s="3"/>
-      <c r="AO3" s="3"/>
-      <c r="AP3" s="3"/>
-      <c r="AQ3" s="3"/>
-      <c r="AR3" s="3"/>
-      <c r="AS3" s="3"/>
-      <c r="AT3" s="3"/>
-      <c r="AU3" s="3"/>
-      <c r="AV3" s="3"/>
-      <c r="AW3" s="3"/>
-      <c r="AX3" s="3"/>
-      <c r="AY3" s="3"/>
-      <c r="AZ3" s="3"/>
-      <c r="BA3" s="3"/>
-      <c r="BB3" s="3"/>
-      <c r="BC3" s="3"/>
-      <c r="BD3" s="3"/>
-      <c r="BE3" s="3"/>
-      <c r="BF3" s="3"/>
+    <row r="3" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+      <c r="AR3" s="4"/>
+      <c r="AS3" s="4"/>
+      <c r="AT3" s="4"/>
+      <c r="AU3" s="4"/>
+      <c r="AV3" s="4"/>
+      <c r="AW3" s="4"/>
+      <c r="AX3" s="4"/>
+      <c r="AY3" s="4"/>
+      <c r="AZ3" s="4"/>
+      <c r="BA3" s="4"/>
+      <c r="BB3" s="4"/>
+      <c r="BC3" s="4"/>
+      <c r="BD3" s="4"/>
+      <c r="BE3" s="4"/>
+      <c r="BF3" s="4"/>
     </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="3"/>
-      <c r="AD4" s="3"/>
-      <c r="AE4" s="3"/>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="3"/>
-      <c r="AH4" s="3"/>
-      <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
-      <c r="AK4" s="3"/>
-      <c r="AL4" s="3"/>
-      <c r="AM4" s="3"/>
-      <c r="AN4" s="3"/>
-      <c r="AO4" s="3"/>
-      <c r="AP4" s="3"/>
-      <c r="AQ4" s="3"/>
-      <c r="AR4" s="3"/>
-      <c r="AS4" s="3"/>
-      <c r="AT4" s="3"/>
-      <c r="AU4" s="3"/>
-      <c r="AV4" s="3"/>
-      <c r="AW4" s="3"/>
-      <c r="AX4" s="3"/>
-      <c r="AY4" s="3"/>
-      <c r="AZ4" s="3"/>
-      <c r="BA4" s="3"/>
-      <c r="BB4" s="3"/>
-      <c r="BC4" s="3"/>
-      <c r="BD4" s="3"/>
-      <c r="BE4" s="3"/>
-      <c r="BF4" s="3"/>
+    <row r="4" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4"/>
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4"/>
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4"/>
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4"/>
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4"/>
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4"/>
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4"/>
+      <c r="AP4" s="4"/>
+      <c r="AQ4" s="4"/>
+      <c r="AR4" s="4"/>
+      <c r="AS4" s="4"/>
+      <c r="AT4" s="4"/>
+      <c r="AU4" s="4"/>
+      <c r="AV4" s="4"/>
+      <c r="AW4" s="4"/>
+      <c r="AX4" s="4"/>
+      <c r="AY4" s="4"/>
+      <c r="AZ4" s="4"/>
+      <c r="BA4" s="4"/>
+      <c r="BB4" s="4"/>
+      <c r="BC4" s="4"/>
+      <c r="BD4" s="4"/>
+      <c r="BE4" s="4"/>
+      <c r="BF4" s="4"/>
     </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="3"/>
-      <c r="AA5" s="3"/>
-      <c r="AB5" s="3"/>
-      <c r="AC5" s="3"/>
-      <c r="AD5" s="3"/>
-      <c r="AE5" s="3"/>
-      <c r="AF5" s="3"/>
-      <c r="AG5" s="3"/>
-      <c r="AH5" s="3"/>
-      <c r="AI5" s="3"/>
-      <c r="AJ5" s="3"/>
-      <c r="AK5" s="3"/>
-      <c r="AL5" s="3"/>
-      <c r="AM5" s="3"/>
-      <c r="AN5" s="3"/>
-      <c r="AO5" s="3"/>
-      <c r="AP5" s="3"/>
-      <c r="AQ5" s="3"/>
-      <c r="AR5" s="3"/>
-      <c r="AS5" s="3"/>
-      <c r="AT5" s="3"/>
-      <c r="AU5" s="3"/>
-      <c r="AV5" s="3"/>
-      <c r="AW5" s="3"/>
-      <c r="AX5" s="3"/>
-      <c r="AY5" s="3"/>
-      <c r="AZ5" s="3"/>
-      <c r="BA5" s="3"/>
-      <c r="BB5" s="3"/>
-      <c r="BC5" s="3"/>
-      <c r="BD5" s="3"/>
-      <c r="BE5" s="3"/>
-      <c r="BF5" s="3"/>
+    <row r="5" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
+      <c r="AF5" s="4"/>
+      <c r="AG5" s="4"/>
+      <c r="AH5" s="4"/>
+      <c r="AI5" s="4"/>
+      <c r="AJ5" s="4"/>
+      <c r="AK5" s="4"/>
+      <c r="AL5" s="4"/>
+      <c r="AM5" s="4"/>
+      <c r="AN5" s="4"/>
+      <c r="AO5" s="4"/>
+      <c r="AP5" s="4"/>
+      <c r="AQ5" s="4"/>
+      <c r="AR5" s="4"/>
+      <c r="AS5" s="4"/>
+      <c r="AT5" s="4"/>
+      <c r="AU5" s="4"/>
+      <c r="AV5" s="4"/>
+      <c r="AW5" s="4"/>
+      <c r="AX5" s="4"/>
+      <c r="AY5" s="4"/>
+      <c r="AZ5" s="4"/>
+      <c r="BA5" s="4"/>
+      <c r="BB5" s="4"/>
+      <c r="BC5" s="4"/>
+      <c r="BD5" s="4"/>
+      <c r="BE5" s="4"/>
+      <c r="BF5" s="4"/>
     </row>
-    <row r="6" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-      <c r="Y6" s="3"/>
-      <c r="Z6" s="3"/>
-      <c r="AA6" s="3"/>
-      <c r="AB6" s="3"/>
-      <c r="AC6" s="3"/>
-      <c r="AD6" s="3"/>
-      <c r="AE6" s="3"/>
-      <c r="AF6" s="3"/>
-      <c r="AG6" s="3"/>
-      <c r="AH6" s="3"/>
-      <c r="AI6" s="3"/>
-      <c r="AJ6" s="3"/>
-      <c r="AK6" s="3"/>
-      <c r="AL6" s="3"/>
-      <c r="AM6" s="3"/>
-      <c r="AN6" s="3"/>
-      <c r="AO6" s="3"/>
-      <c r="AP6" s="3"/>
-      <c r="AQ6" s="3"/>
-      <c r="AR6" s="3"/>
-      <c r="AS6" s="3"/>
-      <c r="AT6" s="3"/>
-      <c r="AU6" s="3"/>
-      <c r="AV6" s="3"/>
-      <c r="AW6" s="3"/>
-      <c r="AX6" s="3"/>
-      <c r="AY6" s="3"/>
-      <c r="AZ6" s="3"/>
-      <c r="BA6" s="3"/>
-      <c r="BB6" s="3"/>
-      <c r="BC6" s="3"/>
-      <c r="BD6" s="3"/>
-      <c r="BE6" s="3"/>
-      <c r="BF6" s="3"/>
+    <row r="6" spans="1:58" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="4"/>
+      <c r="AB6" s="4"/>
+      <c r="AC6" s="4"/>
+      <c r="AD6" s="4"/>
+      <c r="AE6" s="4"/>
+      <c r="AF6" s="4"/>
+      <c r="AG6" s="4"/>
+      <c r="AH6" s="4"/>
+      <c r="AI6" s="4"/>
+      <c r="AJ6" s="4"/>
+      <c r="AK6" s="4"/>
+      <c r="AL6" s="4"/>
+      <c r="AM6" s="4"/>
+      <c r="AN6" s="4"/>
+      <c r="AO6" s="4"/>
+      <c r="AP6" s="4"/>
+      <c r="AQ6" s="4"/>
+      <c r="AR6" s="4"/>
+      <c r="AS6" s="4"/>
+      <c r="AT6" s="4"/>
+      <c r="AU6" s="4"/>
+      <c r="AV6" s="4"/>
+      <c r="AW6" s="4"/>
+      <c r="AX6" s="4"/>
+      <c r="AY6" s="4"/>
+      <c r="AZ6" s="4"/>
+      <c r="BA6" s="4"/>
+      <c r="BB6" s="4"/>
+      <c r="BC6" s="4"/>
+      <c r="BD6" s="4"/>
+      <c r="BE6" s="4"/>
+      <c r="BF6" s="4"/>
     </row>
     <row r="7" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3" t="s">
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-      <c r="Y7" s="3" t="s">
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="4"/>
+      <c r="X7" s="4"/>
+      <c r="Y7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="Z7" s="3"/>
-      <c r="AA7" s="3"/>
-      <c r="AB7" s="3"/>
-      <c r="AC7" s="3"/>
-      <c r="AD7" s="3"/>
-      <c r="AE7" s="3"/>
-      <c r="AF7" s="3"/>
-      <c r="AG7" s="3"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3" t="s">
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="4"/>
+      <c r="AB7" s="4"/>
+      <c r="AC7" s="4"/>
+      <c r="AD7" s="4"/>
+      <c r="AE7" s="4"/>
+      <c r="AF7" s="4"/>
+      <c r="AG7" s="4"/>
+      <c r="AH7" s="4"/>
+      <c r="AI7" s="4"/>
+      <c r="AJ7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="AK7" s="3"/>
-      <c r="AL7" s="3"/>
-      <c r="AM7" s="3"/>
-      <c r="AN7" s="3"/>
-      <c r="AO7" s="3"/>
-      <c r="AP7" s="3"/>
-      <c r="AQ7" s="3"/>
-      <c r="AR7" s="3"/>
-      <c r="AS7" s="3"/>
-      <c r="AT7" s="3"/>
-      <c r="AU7" s="3" t="s">
+      <c r="AK7" s="4"/>
+      <c r="AL7" s="4"/>
+      <c r="AM7" s="4"/>
+      <c r="AN7" s="4"/>
+      <c r="AO7" s="4"/>
+      <c r="AP7" s="4"/>
+      <c r="AQ7" s="4"/>
+      <c r="AR7" s="4"/>
+      <c r="AS7" s="4"/>
+      <c r="AT7" s="4"/>
+      <c r="AU7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AV7" s="3"/>
-      <c r="AW7" s="3"/>
-      <c r="AX7" s="3"/>
-      <c r="AY7" s="3"/>
-      <c r="AZ7" s="3"/>
-      <c r="BA7" s="3"/>
-      <c r="BB7" s="3"/>
-      <c r="BC7" s="3"/>
-      <c r="BD7" s="3"/>
-      <c r="BE7" s="3"/>
+      <c r="AV7" s="4"/>
+      <c r="AW7" s="4"/>
+      <c r="AX7" s="4"/>
+      <c r="AY7" s="4"/>
+      <c r="AZ7" s="4"/>
+      <c r="BA7" s="4"/>
+      <c r="BB7" s="4"/>
+      <c r="BC7" s="4"/>
+      <c r="BD7" s="4"/>
+      <c r="BE7" s="4"/>
     </row>
     <row r="8" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="B8" s="3"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="2">
         <v>1</v>
       </c>
@@ -4428,7 +4428,7 @@
       <c r="AS22" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="AY22" s="4" t="s">
+      <c r="AY22" s="3" t="s">
         <v>503</v>
       </c>
       <c r="BA22" s="2" t="s">

</xml_diff>